<commit_message>
feat: today running creatives from ads tg send implemented
</commit_message>
<xml_diff>
--- a/examples/dima_buyer_20260920.xlsx
+++ b/examples/dima_buyer_20260920.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rt\Work\Tristan\tristan_tools\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D542C3A5-6BF0-42D5-AFBE-F0A68616F1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B07B55-7791-42F4-96A6-714DBF2A599E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="26">
   <si>
     <t>EU</t>
   </si>
@@ -62,49 +62,43 @@
     <t>Крео</t>
   </si>
   <si>
-    <t>UK</t>
-  </si>
-  <si>
-    <t>DACH</t>
-  </si>
-  <si>
     <t>TIR2</t>
   </si>
   <si>
-    <t>IT</t>
-  </si>
-  <si>
-    <t>Великобритания</t>
-  </si>
-  <si>
-    <t>Австрия</t>
-  </si>
-  <si>
-    <t>Хорватия</t>
-  </si>
-  <si>
-    <t>Италия</t>
-  </si>
-  <si>
-    <t>Ирландия</t>
-  </si>
-  <si>
-    <t>Германия</t>
-  </si>
-  <si>
-    <t>Словакия</t>
-  </si>
-  <si>
-    <t>Джерси</t>
-  </si>
-  <si>
-    <t>Дания</t>
-  </si>
-  <si>
-    <t>Чехия</t>
-  </si>
-  <si>
-    <t>Мальта</t>
+    <t>норвегия</t>
+  </si>
+  <si>
+    <t>австрия</t>
+  </si>
+  <si>
+    <t>венгрия</t>
+  </si>
+  <si>
+    <t>чехия</t>
+  </si>
+  <si>
+    <t>словакия</t>
+  </si>
+  <si>
+    <t>германия</t>
+  </si>
+  <si>
+    <t>бельгия</t>
+  </si>
+  <si>
+    <t>дания</t>
+  </si>
+  <si>
+    <t>хорватия</t>
+  </si>
+  <si>
+    <t>нидерланды</t>
+  </si>
+  <si>
+    <t>польша</t>
+  </si>
+  <si>
+    <t>TIR1</t>
   </si>
 </sst>
 </file>
@@ -675,76 +669,114 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE8EB542-02FE-4723-8DCA-736E999494B2}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" style="9" customWidth="1"/>
     <col min="3" max="3" width="13.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="12.5703125" style="9"/>
+    <col min="4" max="16384" width="12.5703125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="8"/>
+    </row>
+    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="B2" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="B3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="8"/>
-    </row>
-    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="B4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="B6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="B7" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="10" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="10" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="10"/>
-    </row>
-    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>